<commit_message>
fix: remover SKU 86136 (QDB BAT SEMIMATE POP ROS) da lista IAF make
Adicionado por engano no commit anterior — não é IAF oficial.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/make_iaf.xlsx
+++ b/data/make_iaf.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2666"/>
+  <dimension ref="A1:C2665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40366,26 +40366,26 @@
     </row>
     <row r="2660">
       <c r="A2660" t="n">
-        <v>86136</v>
+        <v>90668</v>
       </c>
       <c r="B2660" t="inlineStr">
         <is>
-          <t>QDB BAT SEMIMATE POP ROS/SUPREMO 3,6g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 270Q, 30g</t>
         </is>
       </c>
       <c r="C2660" t="inlineStr">
         <is>
-          <t>Quem Disse Berenice</t>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>
     <row r="2661">
       <c r="A2661" t="n">
-        <v>90668</v>
+        <v>90711</v>
       </c>
       <c r="B2661" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 270Q, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 225N, 30g</t>
         </is>
       </c>
       <c r="C2661" t="inlineStr">
@@ -40396,11 +40396,11 @@
     </row>
     <row r="2662">
       <c r="A2662" t="n">
-        <v>90711</v>
+        <v>90716</v>
       </c>
       <c r="B2662" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 225N, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 200N, 30g</t>
         </is>
       </c>
       <c r="C2662" t="inlineStr">
@@ -40411,11 +40411,11 @@
     </row>
     <row r="2663">
       <c r="A2663" t="n">
-        <v>90716</v>
+        <v>90719</v>
       </c>
       <c r="B2663" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 200N, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 180Q, 30g</t>
         </is>
       </c>
       <c r="C2663" t="inlineStr">
@@ -40426,11 +40426,11 @@
     </row>
     <row r="2664">
       <c r="A2664" t="n">
-        <v>90719</v>
+        <v>87819</v>
       </c>
       <c r="B2664" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 180Q, 30g</t>
+          <t>MAKE B BATOM EASY MATE TRUE PLUM, 3,9g</t>
         </is>
       </c>
       <c r="C2664" t="inlineStr">
@@ -40441,29 +40441,14 @@
     </row>
     <row r="2665">
       <c r="A2665" t="n">
-        <v>87819</v>
+        <v>88819</v>
       </c>
       <c r="B2665" t="inlineStr">
         <is>
-          <t>MAKE B BATOM EASY MATE TRUE PLUM, 3,9g</t>
+          <t>QDB GLOSS SONHOS AVELI 4ml</t>
         </is>
       </c>
       <c r="C2665" t="inlineStr">
-        <is>
-          <t>oBoticário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2666">
-      <c r="A2666" t="n">
-        <v>88819</v>
-      </c>
-      <c r="B2666" t="inlineStr">
-        <is>
-          <t>QDB GLOSS SONHOS AVELI 4ml</t>
-        </is>
-      </c>
-      <c r="C2666" t="inlineStr">
         <is>
           <t>Quem Disse Berenice</t>
         </is>

</xml_diff>

<commit_message>
fix: excluir acessórios (pincéis, esponjas, maletas) do IAF make
Acessórios não contam como IAF make pela regra da Boti. Mudanças:

- Heurística is_makeup_product agora exclui PINCEL, ESPONJA, MALETA,
  NECESSAIRE, KIT MAQ
- Remove indicadores ESPONJA MAQ, PINCEL MAQ, MINI MALETA do positivo
- Remove 4 SKUs que eu adicionei por engano em commits anteriores:
  93493 (esponja Eud), 57753 (esponja Make B), 56676 (esponja Niina),
  89568 (mini maleta Make B)

Resultado vs painel: 13706 make gap −1, 13707 make gap 0 (perfeito),
13706 cab gap 0, 13707 cab gap −2. Paletas multifuncionais
(PLT MULTIF, PALETA MULTIF) continuam contando — contêm
sombra/blush/iluminador reais.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/make_iaf.xlsx
+++ b/data/make_iaf.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2665"/>
+  <dimension ref="A1:C2661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40156,26 +40156,26 @@
     </row>
     <row r="2646">
       <c r="A2646" t="n">
-        <v>93493</v>
+        <v>90667</v>
       </c>
       <c r="B2646" t="inlineStr">
         <is>
-          <t>EUD ESPONJA MAQ FAC NIINA SECRETS PU</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 275N, 30g</t>
         </is>
       </c>
       <c r="C2646" t="inlineStr">
         <is>
-          <t>Eudora</t>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>
     <row r="2647">
       <c r="A2647" t="n">
-        <v>90667</v>
+        <v>90709</v>
       </c>
       <c r="B2647" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 275N, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 235N, 30g</t>
         </is>
       </c>
       <c r="C2647" t="inlineStr">
@@ -40186,11 +40186,11 @@
     </row>
     <row r="2648">
       <c r="A2648" t="n">
-        <v>90709</v>
+        <v>90712</v>
       </c>
       <c r="B2648" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 235N, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 220Q, 30g</t>
         </is>
       </c>
       <c r="C2648" t="inlineStr">
@@ -40201,11 +40201,11 @@
     </row>
     <row r="2649">
       <c r="A2649" t="n">
-        <v>90712</v>
+        <v>90720</v>
       </c>
       <c r="B2649" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 220Q, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 175N, 30g</t>
         </is>
       </c>
       <c r="C2649" t="inlineStr">
@@ -40216,11 +40216,11 @@
     </row>
     <row r="2650">
       <c r="A2650" t="n">
-        <v>90720</v>
+        <v>90721</v>
       </c>
       <c r="B2650" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 175N, 30g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 170Q, 30g</t>
         </is>
       </c>
       <c r="C2650" t="inlineStr">
@@ -40231,11 +40231,11 @@
     </row>
     <row r="2651">
       <c r="A2651" t="n">
-        <v>90721</v>
+        <v>87818</v>
       </c>
       <c r="B2651" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 170Q, 30g</t>
+          <t>MAKE B BATOM EASY MATE WHISPER BEIGE, 3,9g</t>
         </is>
       </c>
       <c r="C2651" t="inlineStr">
@@ -40246,11 +40246,11 @@
     </row>
     <row r="2652">
       <c r="A2652" t="n">
-        <v>87818</v>
+        <v>87820</v>
       </c>
       <c r="B2652" t="inlineStr">
         <is>
-          <t>MAKE B BATOM EASY MATE WHISPER BEIGE, 3,9g</t>
+          <t>MAKE B BATOM EASY MATE WARM CLAY, 3,9g</t>
         </is>
       </c>
       <c r="C2652" t="inlineStr">
@@ -40261,11 +40261,11 @@
     </row>
     <row r="2653">
       <c r="A2653" t="n">
-        <v>87820</v>
+        <v>87787</v>
       </c>
       <c r="B2653" t="inlineStr">
         <is>
-          <t>MAKE B BATOM EASY MATE WARM CLAY, 3,9g</t>
+          <t>MAKE B PLT MULTIF BL/FUS SOFT FUSION 20g</t>
         </is>
       </c>
       <c r="C2653" t="inlineStr">
@@ -40276,41 +40276,41 @@
     </row>
     <row r="2654">
       <c r="A2654" t="n">
-        <v>57753</v>
+        <v>89085</v>
       </c>
       <c r="B2654" t="inlineStr">
         <is>
-          <t>MAKE B ESPONJA MAQ PU</t>
+          <t>NIINA SECRETS GLOSS LABIAL LUMINOUS SUMMER COR 2 12g</t>
         </is>
       </c>
       <c r="C2654" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
     <row r="2655">
       <c r="A2655" t="n">
-        <v>89568</v>
+        <v>95702</v>
       </c>
       <c r="B2655" t="inlineStr">
         <is>
-          <t>MAKE B MINI MALETA ALL SET</t>
+          <t>COMB NIINA SCRT NEUTRALS NAM/26</t>
         </is>
       </c>
       <c r="C2655" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
     <row r="2656">
       <c r="A2656" t="n">
-        <v>87787</v>
+        <v>90668</v>
       </c>
       <c r="B2656" t="inlineStr">
         <is>
-          <t>MAKE B PLT MULTIF BL/FUS SOFT FUSION 20g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 270Q, 30g</t>
         </is>
       </c>
       <c r="C2656" t="inlineStr">
@@ -40321,56 +40321,56 @@
     </row>
     <row r="2657">
       <c r="A2657" t="n">
-        <v>89085</v>
+        <v>90711</v>
       </c>
       <c r="B2657" t="inlineStr">
         <is>
-          <t>NIINA SECRETS GLOSS LABIAL LUMINOUS SUMMER COR 2 12g</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 225N, 30g</t>
         </is>
       </c>
       <c r="C2657" t="inlineStr">
         <is>
-          <t>Eudora</t>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>
     <row r="2658">
       <c r="A2658" t="n">
-        <v>95702</v>
+        <v>90716</v>
       </c>
       <c r="B2658" t="inlineStr">
         <is>
-          <t>COMB NIINA SCRT NEUTRALS NAM/26</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 200N, 30g</t>
         </is>
       </c>
       <c r="C2658" t="inlineStr">
         <is>
-          <t>Eudora</t>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>
     <row r="2659">
       <c r="A2659" t="n">
-        <v>56676</v>
+        <v>90719</v>
       </c>
       <c r="B2659" t="inlineStr">
         <is>
-          <t>NIINA REPACK ESPONJA DE MAKE</t>
+          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 180Q, 30g</t>
         </is>
       </c>
       <c r="C2659" t="inlineStr">
         <is>
-          <t>Eudora</t>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>
     <row r="2660">
       <c r="A2660" t="n">
-        <v>90668</v>
+        <v>87819</v>
       </c>
       <c r="B2660" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 270Q, 30g</t>
+          <t>MAKE B BATOM EASY MATE TRUE PLUM, 3,9g</t>
         </is>
       </c>
       <c r="C2660" t="inlineStr">
@@ -40381,74 +40381,14 @@
     </row>
     <row r="2661">
       <c r="A2661" t="n">
-        <v>90711</v>
+        <v>88819</v>
       </c>
       <c r="B2661" t="inlineStr">
         <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 225N, 30g</t>
+          <t>QDB GLOSS SONHOS AVELI 4ml</t>
         </is>
       </c>
       <c r="C2661" t="inlineStr">
-        <is>
-          <t>oBoticário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2662">
-      <c r="A2662" t="n">
-        <v>90716</v>
-      </c>
-      <c r="B2662" t="inlineStr">
-        <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 200N, 30g</t>
-        </is>
-      </c>
-      <c r="C2662" t="inlineStr">
-        <is>
-          <t>oBoticário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2663">
-      <c r="A2663" t="n">
-        <v>90719</v>
-      </c>
-      <c r="B2663" t="inlineStr">
-        <is>
-          <t>MAKE B BASE LÍQUIDA MATE SALICYLIC 180Q, 30g</t>
-        </is>
-      </c>
-      <c r="C2663" t="inlineStr">
-        <is>
-          <t>oBoticário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2664">
-      <c r="A2664" t="n">
-        <v>87819</v>
-      </c>
-      <c r="B2664" t="inlineStr">
-        <is>
-          <t>MAKE B BATOM EASY MATE TRUE PLUM, 3,9g</t>
-        </is>
-      </c>
-      <c r="C2664" t="inlineStr">
-        <is>
-          <t>oBoticário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2665">
-      <c r="A2665" t="n">
-        <v>88819</v>
-      </c>
-      <c r="B2665" t="inlineStr">
-        <is>
-          <t>QDB GLOSS SONHOS AVELI 4ml</t>
-        </is>
-      </c>
-      <c r="C2665" t="inlineStr">
         <is>
           <t>Quem Disse Berenice</t>
         </is>

</xml_diff>